<commit_message>
Hand jig flipper commands to the robot so the pendant can flip and jog.
A missed jig-placed prox times out back to wait, and releasing E-stop does not restart the cycle.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/machines/big_jig_flipper/wiring.xlsx
+++ b/machines/big_jig_flipper/wiring.xlsx
@@ -10,12 +10,14 @@
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Outputs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Robot" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inputs'!$A$6:$F$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Inputs'!$6:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outputs'!$A$6:$F$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Outputs'!$6:$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Robot'!$A$4:$D$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +69,10 @@
     <font>
       <name val="Arial"/>
       <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -152,6 +158,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -857,24 +875,24 @@
           <t>X109</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Robot</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Robot jig-placed</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Jig placed</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Jig fully placed prox</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>JigPlaced</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Robot says the jig is set. After set-down has settled, the clamps are allowed to open.</t>
+          <t>Jig is fully placed. After set-down settles, the clamps may open. If this stays off for 40 seconds, the cycle faults and returns to wait.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1097,7 +1115,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Valves on the bottom of the Click Y2 module. Every output is off on E-stop, and off while only waiting in C1.</t>
+          <t>Allow jig sense is Y206. Valves follow on Y207-Y216. Every output is off on E-stop, and off while only waiting in C1.</t>
         </is>
       </c>
     </row>
@@ -1281,22 +1299,22 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Head-stock lift</t>
+          <t>Robot</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Head-stock lift up valve</t>
+          <t>Allow jig sense</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Lift1UpValve</t>
+          <t>AllowJigSense</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Lifts the head stock until its up prox. Auto while that side is lifting and not setting down. Jog: lift-1 up. Off on E-stop.</t>
+          <t>Enables jig sensing during set-down. Off while waiting in hold. Off on E-stop.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1318,17 +1336,17 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Head-stock lift down valve</t>
+          <t>Head-stock lift up valve</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Lift1DnValve</t>
+          <t>Lift1UpValve</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Lowers the head stock during set-down, or on jog lift-1 down. Stays off while waiting in hold. Off on E-stop.</t>
+          <t>Lifts the head stock until its up prox. Auto while that side is lifting and not setting down. Jog: lift-1 up. Off on E-stop.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1345,22 +1363,22 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Tail-stock lift</t>
+          <t>Head-stock lift</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Tail-stock lift up valve</t>
+          <t>Head-stock lift down valve</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Lift2UpValve</t>
+          <t>Lift1DnValve</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Lifts the tail stock until its own up prox. Does not drop when the head stock arrives first. Off on E-stop.</t>
+          <t>Lowers the head stock during set-down, or on jog lift-1 down. Stays off while waiting in hold. Off on E-stop.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1382,17 +1400,17 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Tail-stock lift down valve</t>
+          <t>Tail-stock lift up valve</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Lift2DnValve</t>
+          <t>Lift2UpValve</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Lowers the tail stock during set-down, or on jog lift-2 down. Stays off while waiting in hold. Off on E-stop.</t>
+          <t>Lifts the tail stock until its own up prox. Does not drop when the head stock arrives first. Off on E-stop.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1409,22 +1427,22 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Head-stock clamp</t>
+          <t>Tail-stock lift</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Head-stock clamp-in valve</t>
+          <t>Tail-stock lift down valve</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Clamp1Valve</t>
+          <t>Lift2DnValve</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Closes the head clamp until the clamped prox. Jog: clamp-1 in. Off on E-stop.</t>
+          <t>Lowers the tail stock during set-down, or on jog lift-2 down. Stays off while waiting in hold. Off on E-stop.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1446,17 +1464,17 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Head-stock unclamp valve</t>
+          <t>Head-stock clamp-in valve</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Unclamp1Valve</t>
+          <t>Clamp1Valve</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Opens the head clamp until the unclamped prox. Jog: clamp-1 out. Off on E-stop.</t>
+          <t>Closes the head clamp until the clamped prox. Jog: clamp-1 in. Off on E-stop.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1473,22 +1491,22 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Tail-stock clamp</t>
+          <t>Head-stock clamp</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Tail-stock clamp-in valve</t>
+          <t>Head-stock unclamp valve</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Clamp2Valve</t>
+          <t>Unclamp1Valve</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Closes the tail clamp until the clamped prox. Jog: clamp-2 in. Off on E-stop.</t>
+          <t>Opens the head clamp until the unclamped prox. Jog: clamp-1 out. Off on E-stop.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1510,17 +1528,17 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Tail-stock unclamp valve</t>
+          <t>Tail-stock clamp-in valve</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Unclamp2Valve</t>
+          <t>Clamp2Valve</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Opens the tail clamp until the unclamped prox. Jog: clamp-2 out. Off on E-stop.</t>
+          <t>Closes the tail clamp until the clamped prox. Jog: clamp-2 in. Off on E-stop.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1537,22 +1555,22 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Rotate</t>
+          <t>Tail-stock clamp</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Rotate to A valve</t>
+          <t>Tail-stock unclamp valve</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>RotateToAValve</t>
+          <t>Unclamp2Valve</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Rotates toward A. Both clamped proxes (X103 and X104) must be on. Jog: rotate A. Off on E-stop.</t>
+          <t>Opens the tail clamp until the unclamped prox. Jog: clamp-2 out. Off on E-stop.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1574,17 +1592,17 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Rotate to B valve</t>
+          <t>Rotate to A valve</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>RotateToBValve</t>
+          <t>RotateToAValve</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Rotates toward B. Both clamped proxes (X103 and X104) must be on. Jog: rotate B. Off on E-stop.</t>
+          <t>Rotates toward A. Both clamped proxes (X103 and X104) must be on. Jog: rotate A. Off on E-stop.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1601,22 +1619,22 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Robot</t>
+          <t>Rotate</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Allow jig sense</t>
+          <t>Rotate to B valve</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>AllowJigSense</t>
+          <t>RotateToBValve</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Enables jig sensing during set-down. Off while waiting in hold. Off on E-stop.</t>
+          <t>Rotates toward B. Both clamped proxes (X103 and X104) must be on. Jog: rotate B. Off on E-stop.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1672,7 +1690,7 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>machines/big_jig_flipper address map. Side 1 is the head stock. Side 2 is the tail stock.</t>
+          <t>machines/big_jig_flipper address map. Side 1 is the head stock. Side 2 is the tail stock. Robot words are on the Robot sheet.</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1702,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>X101–X116. Nine sensors are used. X110–X116 are open.</t>
+          <t>X101-X116. Nine points are used. X109 is the jig-fully-placed prox. X110-X116 are open.</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1714,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Y201–Y216. Valves are wired on the bottom, Y206–Y216. Y201–Y205 are open.</t>
+          <t>Y201-Y216. Allow jig sense is Y206. Valves follow on Y207-Y216. Y201-Y205 are open.</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1750,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>C21 is jog mode. C22–C31 are the jog pushes. A jog command can still energize its valve while C1 is on.</t>
+          <t>Pendant jog is DS9-DS20. DS9 is jog mode. DS10-DS13 are the lift buttons. DS20 links both lifts so one up button raises both and one down button lowers both. Leave DS20 at 0 for independent lifts. DS14-DS19 are clamps and rotate. E-stop still drops the valve.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1762,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Y214 and Y215 also require both clamped proxes, X103 and X104.</t>
+          <t>Y215 and Y216 also require both clamped proxes, X103 and X104.</t>
         </is>
       </c>
     </row>
@@ -1767,4 +1785,505 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Big jig flipper robot words</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Click is the EtherNet/IP adapter. DS1-DS4 go to the YRC1000 scanner. DS5-DS20 come from the scanner. Each word is 0 or 1. Extend the Click assembly so the from-scanner block covers DS5 through DS20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>DS1</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>To scanner</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>1 while the machine is in wait and there is no place error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>DS2</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>To scanner</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Place error</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>1 when the jig is not placed within 40 seconds of set-down. Stays 1 until DS8 acknowledges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>DS3</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>To scanner</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>At A</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>1 while the A position prox is on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>DS4</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>To scanner</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>At B</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>1 while the B position prox is on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>DS5</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Flip to A</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Any non-zero value asks for a flip to A. Ignored when the jig is already at A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>DS6</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Flip to B</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Any non-zero value asks for a flip to B. Ignored when the jig is already at B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>DS7</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Spare</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Open. Jig placed is the X109 prox, not a robot word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>DS8</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Error acknowledge</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Any non-zero value clears the place error and lets DS1 go ready again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>DS9</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Jog mode</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Any non-zero value enables jog. Auto valves stay off while this is on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>DS10</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Jog head lift up</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Jog the head-stock lift up. Needs jog mode. With DS20 on, this also raises the tail stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>DS11</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Jog head lift down</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Jog the head-stock lift down. Needs jog mode. With DS20 on, this also lowers the tail stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>DS12</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Jog tail lift up</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Jog the tail-stock lift up. Needs jog mode. With DS20 on, this also raises the head stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>DS13</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Jog tail lift down</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Jog the tail-stock lift down. Needs jog mode. With DS20 on, this also lowers the head stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>DS14</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Jog head clamp in</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Jog the head-stock clamp in. Needs jog mode. Opposed with DS15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>DS15</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Jog head unclamp</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Jog the head-stock unclamp. Needs jog mode. Opposed with DS14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>DS16</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Jog tail clamp in</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Jog the tail-stock clamp in. Needs jog mode. Opposed with DS17.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>DS17</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Jog tail unclamp</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Jog the tail-stock unclamp. Needs jog mode. Opposed with DS16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>DS18</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Jog rotate to A</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Jog rotate toward A. Needs jog mode and both clamped proxes. Opposed with DS19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>DS19</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Jog rotate to B</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Jog rotate toward B. Needs jog mode and both clamped proxes. Opposed with DS18.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>DS20</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>From scanner</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Link lifts</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Any non-zero value links the lifts. One up button raises both sides. One down button lowers both. Leave at 0 for independent jog.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:D24"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>